<commit_message>
refactor(debug): make LiDAR diagnostics configurable
Add a compile-time LIDAR_DIAGNOSTICS switch.
- Exclude diagnostic counters and buffer snapshots when disabled.
Preserve USART3 DMA reception, error recovery, packet parsing,
and RPM calculation in both configurations.
</commit_message>
<xml_diff>
--- a/STM32F407 PIN CONFIG MAP.xlsx
+++ b/STM32F407 PIN CONFIG MAP.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Programing_Files_IoT\STM32CubeIDE\workspace_2.1.1\STM32F407VET6\Moppy2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{82764778-BEA1-43E7-8E65-228532243539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A396D814-9B9B-4EF5-AEF0-0A2B3926265C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9060" windowWidth="15990" windowHeight="24990" xr2:uid="{305A6F52-E2CA-4EBC-B1AC-84056AC3DA93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{305A6F52-E2CA-4EBC-B1AC-84056AC3DA93}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="PinOut" sheetId="1" r:id="rId1"/>
+    <sheet name="Power Consumption" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="131">
   <si>
     <t>3V3</t>
   </si>
@@ -397,13 +397,46 @@
   </si>
   <si>
     <t>I2C3/SDA</t>
+  </si>
+  <si>
+    <t>USART3_RX</t>
+  </si>
+  <si>
+    <t>USART3_TX</t>
+  </si>
+  <si>
+    <t>LiDar_TX</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Signal Type</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>RPM</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>mA</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Lidar Motor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -418,8 +451,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,6 +545,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -584,7 +637,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -690,6 +743,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1043,7 +1108,7 @@
     <col min="12" max="12" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1057,7 +1122,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1071,7 +1136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C5" s="14" t="s">
         <v>1</v>
       </c>
@@ -1085,7 +1150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>90</v>
       </c>
@@ -1105,7 +1170,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>41</v>
       </c>
@@ -1125,7 +1190,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
         <v>93</v>
       </c>
@@ -1151,7 +1216,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>100</v>
       </c>
@@ -1177,7 +1242,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>87</v>
       </c>
@@ -1197,7 +1262,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
@@ -1211,7 +1276,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C12" s="24" t="s">
         <v>15</v>
       </c>
@@ -1225,7 +1290,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>96</v>
       </c>
@@ -1245,7 +1310,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="28" t="s">
         <v>101</v>
       </c>
@@ -1264,14 +1329,23 @@
       <c r="F14" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="H14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="37" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K14" t="s">
+        <v>120</v>
+      </c>
+      <c r="L14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
         <v>112</v>
       </c>
@@ -1297,7 +1371,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
         <v>104</v>
       </c>
@@ -1538,6 +1612,364 @@
       <c r="E29" s="2" t="s">
         <v>88</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B338E491-708B-463B-A1C3-4420A61255C7}">
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" style="27" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>126</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="39" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="3">
+        <v>300</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3">
+        <v>55</v>
+      </c>
+      <c r="G2" s="3">
+        <f>SUM(E2*F2/1000)</f>
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="40"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="40"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="40"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="40"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="40"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="40"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="40"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="40"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="40"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Before FreeRTOS: IMU configurations on going
</commit_message>
<xml_diff>
--- a/STM32F407 PIN CONFIG MAP.xlsx
+++ b/STM32F407 PIN CONFIG MAP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Programing_Files_IoT\STM32CubeIDE\workspace_2.1.1\STM32F407VET6\Moppy2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A396D814-9B9B-4EF5-AEF0-0A2B3926265C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCABEFF-D63E-4ADF-9356-9F5626728F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{305A6F52-E2CA-4EBC-B1AC-84056AC3DA93}"/>
+    <workbookView xWindow="28680" yWindow="-9060" windowWidth="15990" windowHeight="24990" activeTab="1" xr2:uid="{305A6F52-E2CA-4EBC-B1AC-84056AC3DA93}"/>
   </bookViews>
   <sheets>
     <sheet name="PinOut" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="132">
   <si>
     <t>3V3</t>
   </si>
@@ -430,6 +430,9 @@
   </si>
   <si>
     <t>Lidar Motor</t>
+  </si>
+  <si>
+    <t>ALL 6</t>
   </si>
 </sst>
 </file>
@@ -1681,7 +1684,10 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="G3" s="3">
+        <f t="shared" ref="G3:G12" si="0">SUM(E3*F3/1000)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="40"/>
@@ -1690,7 +1696,10 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="G4" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
@@ -1699,7 +1708,10 @@
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="40"/>
@@ -1708,7 +1720,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="G6" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="40"/>
@@ -1717,7 +1732,10 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="40"/>
@@ -1726,7 +1744,10 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="40"/>
@@ -1735,7 +1756,10 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="G9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="40"/>
@@ -1744,7 +1768,10 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="40"/>
@@ -1753,16 +1780,32 @@
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
+      <c r="G11" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
+      <c r="A12" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="6">
+        <v>900</v>
+      </c>
       <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="E12" s="6">
+        <v>12</v>
+      </c>
+      <c r="F12" s="6">
+        <v>494</v>
+      </c>
+      <c r="G12" s="3">
+        <f t="shared" si="0"/>
+        <v>5.9279999999999999</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>

</xml_diff>

<commit_message>
feat(rtos): add dedicated tasks and motion command support
- Add dedicated IMU, wheel control, general control, and telemetry tasks.
- Move IMU processing into ImuTask.
- Run chassis control periodically in WheelTask at 20 ms intervals.
- Add motion command support for forward/reverse movement and adjustable left/right turning.
- Support differential-drive wheel speed targets for coordinated movement.
- Move chassis timing diagnostics into WheelTask.
- Keep button handling, brush control, LiDAR PID, and OLED updates in GeneralTask.
- Initialize robot peripherals before starting the RTOS scheduler.
- Prepare TelemetryTask for Raspberry Pi communication and navigation commands.
- Maintain watchdog servicing during general control execution.
</commit_message>
<xml_diff>
--- a/STM32F407 PIN CONFIG MAP.xlsx
+++ b/STM32F407 PIN CONFIG MAP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Programing_Files_IoT\STM32CubeIDE\workspace_2.1.1\STM32F407VET6\Moppy2.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCABEFF-D63E-4ADF-9356-9F5626728F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37816DA-8021-4E0E-8212-F9C461ABCDFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9060" windowWidth="15990" windowHeight="24990" activeTab="1" xr2:uid="{305A6F52-E2CA-4EBC-B1AC-84056AC3DA93}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{305A6F52-E2CA-4EBC-B1AC-84056AC3DA93}"/>
   </bookViews>
   <sheets>
     <sheet name="PinOut" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="132">
   <si>
     <t>3V3</t>
   </si>
@@ -1097,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6FA93B-C689-410F-8E49-03A0B06E9A5F}">
-  <dimension ref="A3:L29"/>
+  <dimension ref="A3:R29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" style="1" customWidth="1"/>
@@ -1111,7 +1111,7 @@
     <col min="12" max="12" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1139,7 +1139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C5" s="14" t="s">
         <v>1</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>90</v>
       </c>
@@ -1173,7 +1173,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>41</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
         <v>93</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>100</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>87</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C12" s="24" t="s">
         <v>15</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>96</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="28" t="s">
         <v>101</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
         <v>112</v>
       </c>
@@ -1373,8 +1373,11 @@
       <c r="J15" s="8" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="R15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
         <v>104</v>
       </c>

</xml_diff>